<commit_message>
Tambah bahan dan edit susunan acara
</commit_message>
<xml_diff>
--- a/0. Rundown RKT.xlsx
+++ b/0. Rundown RKT.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="22527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ASATIDZ\Zen\persiapan-rkt-2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MABAIZ\Persiapan RKT 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67F4FEDC-AD53-4678-9209-70CB7BE13ABD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD2F776C-950D-4564-A28A-215ABE671106}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19455" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -20,12 +20,7 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -33,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="56">
   <si>
     <t>RAPAT KERJA TAHUNAN (RKT) GABUNGAN</t>
   </si>
@@ -208,6 +203,12 @@
 - Tahfidz (berapa banyak juziyah dan syahadah santri)
 - Tahsin (berapa banyak yang belum lancar tahsinnya dalam waktu setahun)
 - Aspirasi</t>
+  </si>
+  <si>
+    <t>Tilawah Al-Quran</t>
+  </si>
+  <si>
+    <t>Ust. Ahmad Yudha Nugraha, S.Pd.</t>
   </si>
 </sst>
 </file>
@@ -270,10 +271,10 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -550,7 +551,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="11.7109375" style="1" customWidth="1"/>
@@ -562,40 +563,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
     </row>
     <row r="3" spans="1:4">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
+      <c r="B3" s="4"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
     </row>
     <row r="5" spans="1:4">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="4"/>
+      <c r="B5" s="5"/>
     </row>
     <row r="6" spans="1:4">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="4"/>
+      <c r="B6" s="5"/>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="2" t="s">
@@ -624,220 +625,230 @@
       <c r="D9" s="2"/>
     </row>
     <row r="10" spans="1:4" ht="30">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="2"/>
+      <c r="B10" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D10" s="2"/>
+    </row>
+    <row r="11" spans="1:4" ht="30">
+      <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B11" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C11" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D10" s="2"/>
-    </row>
-    <row r="11" spans="1:4">
-      <c r="A11" s="2" t="s">
+      <c r="D11" s="2"/>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B12" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C12" s="2" t="s">
         <v>17</v>
-      </c>
-      <c r="D11" s="2"/>
-    </row>
-    <row r="12" spans="1:4" ht="30">
-      <c r="A12" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>20</v>
       </c>
       <c r="D12" s="2"/>
     </row>
     <row r="13" spans="1:4" ht="30">
       <c r="A13" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" s="2"/>
+    </row>
+    <row r="14" spans="1:4" ht="30">
+      <c r="A14" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B14" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C14" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D13" s="2"/>
-    </row>
-    <row r="14" spans="1:4">
-      <c r="A14" s="2" t="s">
+      <c r="D14" s="2"/>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B15" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C15" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D14" s="2"/>
-    </row>
-    <row r="15" spans="1:4" ht="30">
-      <c r="A15" s="2" t="s">
+      <c r="D15" s="2"/>
+    </row>
+    <row r="16" spans="1:4" ht="30">
+      <c r="A16" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B16" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C16" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D15" s="2"/>
-    </row>
-    <row r="16" spans="1:4">
-      <c r="A16" s="2" t="s">
+      <c r="D16" s="2"/>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B17" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C17" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D16" s="2"/>
-    </row>
-    <row r="17" spans="1:5" ht="30">
-      <c r="A17" s="2" t="s">
+      <c r="D17" s="2"/>
+    </row>
+    <row r="18" spans="1:5" ht="30">
+      <c r="A18" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B18" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C18" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D17" s="2"/>
-      <c r="E17" s="1" t="s">
+      <c r="D18" s="2"/>
+      <c r="E18" s="1" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="105">
-      <c r="A18" s="2" t="s">
+    <row r="19" spans="1:5" ht="105">
+      <c r="A19" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B19" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="C19" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="D19" s="2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="45">
-      <c r="A19" s="2" t="s">
+    <row r="20" spans="1:5" ht="45">
+      <c r="A20" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B20" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="C20" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="D20" s="2" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
-      <c r="A20" s="2" t="s">
+    <row r="21" spans="1:5">
+      <c r="A21" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B21" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="C21" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D20" s="2"/>
-    </row>
-    <row r="21" spans="1:5" ht="135">
-      <c r="A21" s="2" t="s">
+      <c r="D21" s="2"/>
+    </row>
+    <row r="22" spans="1:5" ht="135">
+      <c r="A22" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B22" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C22" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="D21" s="2"/>
-    </row>
-    <row r="22" spans="1:5">
-      <c r="A22" s="2" t="s">
+      <c r="D22" s="2"/>
+    </row>
+    <row r="23" spans="1:5">
+      <c r="A23" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B23" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C23" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D22" s="2"/>
-    </row>
-    <row r="24" spans="1:5">
-      <c r="A24" s="4" t="s">
+      <c r="D23" s="2"/>
+    </row>
+    <row r="25" spans="1:5">
+      <c r="A25" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="B24" s="4"/>
-      <c r="C24" s="4"/>
-      <c r="D24" s="4"/>
-    </row>
-    <row r="25" spans="1:5">
-      <c r="A25" s="4" t="s">
+      <c r="B25" s="5"/>
+      <c r="C25" s="5"/>
+      <c r="D25" s="5"/>
+    </row>
+    <row r="26" spans="1:5">
+      <c r="A26" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="B25" s="4"/>
-      <c r="C25" s="4"/>
-      <c r="D25" s="4"/>
-    </row>
-    <row r="26" spans="1:5">
-      <c r="A26" s="4" t="s">
+      <c r="B26" s="5"/>
+      <c r="C26" s="5"/>
+      <c r="D26" s="5"/>
+    </row>
+    <row r="27" spans="1:5">
+      <c r="A27" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="B26" s="4"/>
-      <c r="C26" s="4"/>
-      <c r="D26" s="4"/>
-    </row>
-    <row r="27" spans="1:5">
-      <c r="A27" s="4" t="s">
+      <c r="B27" s="5"/>
+      <c r="C27" s="5"/>
+      <c r="D27" s="5"/>
+    </row>
+    <row r="28" spans="1:5">
+      <c r="A28" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="B27" s="4"/>
-      <c r="C27" s="4"/>
-      <c r="D27" s="4"/>
-    </row>
-    <row r="28" spans="1:5">
-      <c r="A28" s="4" t="s">
+      <c r="B28" s="5"/>
+      <c r="C28" s="5"/>
+      <c r="D28" s="5"/>
+    </row>
+    <row r="29" spans="1:5">
+      <c r="A29" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="B28" s="4"/>
-      <c r="C28" s="4"/>
-      <c r="D28" s="4"/>
+      <c r="B29" s="5"/>
+      <c r="C29" s="5"/>
+      <c r="D29" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="A29:D29"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A24:D24"/>
-    <mergeCell ref="A25:D25"/>
-    <mergeCell ref="A26:D26"/>
-    <mergeCell ref="A27:D27"/>
-    <mergeCell ref="A28:D28"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>